<commit_message>
updated BGDP to world bank source
</commit_message>
<xml_diff>
--- a/InputData/io-model/BGDP/BAU GDP.xlsx
+++ b/InputData/io-model/BGDP/BAU GDP.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\io-model\BGDP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE03504-E93D-4FB9-94DA-02C444102EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF8980EE-C492-4D21-94DA-D296506377A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="OECD Data MEX" sheetId="6" r:id="rId2"/>
-    <sheet name="BGDP" sheetId="2" r:id="rId3"/>
+    <sheet name="world bank data" sheetId="7" r:id="rId3"/>
+    <sheet name="BGDP" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>BGDP BAU Gross Domestic Product</t>
   </si>
@@ -58,9 +59,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>The OECD long-term forecast gives GDPs in millions of 2015 USD with Purchasing Power Parity.</t>
-  </si>
-  <si>
     <t>In the U.S. model, input data are converted to 2012 USD (then converted to the</t>
   </si>
   <si>
@@ -86,13 +84,49 @@
   </si>
   <si>
     <t>GDP</t>
+  </si>
+  <si>
+    <t>Country Name</t>
+  </si>
+  <si>
+    <t>Country Code</t>
+  </si>
+  <si>
+    <t>Indicator Name</t>
+  </si>
+  <si>
+    <t>Indicator Code</t>
+  </si>
+  <si>
+    <t>MEX</t>
+  </si>
+  <si>
+    <t>GDP (constant 2015 US$)</t>
+  </si>
+  <si>
+    <t>NY.GDP.MKTP.KD</t>
+  </si>
+  <si>
+    <t>World Bank Group</t>
+  </si>
+  <si>
+    <t>https://data.worldbank.org/indicator/NY.GDP.MKTP.KD?locations=MX</t>
+  </si>
+  <si>
+    <t>GDP (constant 2015 US$) - Mexico</t>
+  </si>
+  <si>
+    <t>The world bank long-term forecast gives GDPs in millions of 2015 USD</t>
+  </si>
+  <si>
+    <t>2012 USD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,13 +170,26 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -154,11 +201,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -179,10 +227,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -460,80 +514,92 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="77.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D4" s="2">
         <v>2023</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>0.9686815713640794</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <f>10^6</f>
         <v>1000000</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D5" r:id="rId1" xr:uid="{AEA3AB9E-B33F-4D38-8574-2CC72EBFA909}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -563,16 +629,16 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="9"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>12</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>13</v>
       </c>
       <c r="G3" s="5"/>
     </row>
@@ -591,6 +657,10 @@
       <c r="B5" s="10">
         <v>2350000000000</v>
       </c>
+      <c r="C5" s="13">
+        <f>B5/$B$4</f>
+        <v>1.0585585585585586</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
@@ -599,6 +669,10 @@
       <c r="B6" s="10">
         <v>2450000000000</v>
       </c>
+      <c r="C6" s="13">
+        <f t="shared" ref="C6:C44" si="0">B6/$B$4</f>
+        <v>1.1036036036036037</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
@@ -607,6 +681,10 @@
       <c r="B7" s="10">
         <v>2530000000000</v>
       </c>
+      <c r="C7" s="13">
+        <f t="shared" si="0"/>
+        <v>1.1396396396396395</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
@@ -615,6 +693,10 @@
       <c r="B8" s="10">
         <v>2590000000000</v>
       </c>
+      <c r="C8" s="13">
+        <f t="shared" si="0"/>
+        <v>1.1666666666666667</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
@@ -623,6 +705,10 @@
       <c r="B9" s="10">
         <v>2650000000000</v>
       </c>
+      <c r="C9" s="13">
+        <f t="shared" si="0"/>
+        <v>1.1936936936936937</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
@@ -631,6 +717,10 @@
       <c r="B10" s="10">
         <v>2710000000000</v>
       </c>
+      <c r="C10" s="13">
+        <f t="shared" si="0"/>
+        <v>1.2207207207207207</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
@@ -639,6 +729,10 @@
       <c r="B11" s="10">
         <v>2790000000000</v>
       </c>
+      <c r="C11" s="13">
+        <f t="shared" si="0"/>
+        <v>1.2567567567567568</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
@@ -647,6 +741,10 @@
       <c r="B12" s="10">
         <v>2860000000000</v>
       </c>
+      <c r="C12" s="13">
+        <f t="shared" si="0"/>
+        <v>1.2882882882882882</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
@@ -655,6 +753,10 @@
       <c r="B13" s="10">
         <v>2940000000000</v>
       </c>
+      <c r="C13" s="13">
+        <f t="shared" si="0"/>
+        <v>1.3243243243243243</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
@@ -663,6 +765,10 @@
       <c r="B14" s="10">
         <v>3030000000000</v>
       </c>
+      <c r="C14" s="13">
+        <f t="shared" si="0"/>
+        <v>1.3648648648648649</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
@@ -671,6 +777,10 @@
       <c r="B15" s="10">
         <v>3120000000000</v>
       </c>
+      <c r="C15" s="13">
+        <f t="shared" si="0"/>
+        <v>1.4054054054054055</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
@@ -679,241 +789,357 @@
       <c r="B16" s="10">
         <v>3210000000000</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" s="13">
+        <f t="shared" si="0"/>
+        <v>1.4459459459459461</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>2033</v>
       </c>
       <c r="B17" s="10">
         <v>3300000000000</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" s="13">
+        <f t="shared" si="0"/>
+        <v>1.4864864864864864</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>2034</v>
       </c>
       <c r="B18" s="10">
         <v>3400000000000</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" s="13">
+        <f t="shared" si="0"/>
+        <v>1.5315315315315314</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>2035</v>
       </c>
       <c r="B19" s="10">
         <v>3510000000000</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" s="13">
+        <f t="shared" si="0"/>
+        <v>1.5810810810810811</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9">
         <v>2036</v>
       </c>
       <c r="B20" s="10">
         <v>3610000000000</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" s="13">
+        <f t="shared" si="0"/>
+        <v>1.6261261261261262</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>2037</v>
       </c>
       <c r="B21" s="10">
         <v>3720000000000</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" s="13">
+        <f t="shared" si="0"/>
+        <v>1.6756756756756757</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>2038</v>
       </c>
       <c r="B22" s="10">
         <v>3840000000000</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" s="13">
+        <f t="shared" si="0"/>
+        <v>1.7297297297297298</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>2039</v>
       </c>
       <c r="B23" s="10">
         <v>3950000000000</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" s="13">
+        <f t="shared" si="0"/>
+        <v>1.7792792792792793</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>2040</v>
       </c>
       <c r="B24" s="10">
         <v>4070000000000</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" s="13">
+        <f t="shared" si="0"/>
+        <v>1.8333333333333333</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>2041</v>
       </c>
       <c r="B25" s="10">
         <v>4190000000000</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C25" s="13">
+        <f t="shared" si="0"/>
+        <v>1.8873873873873874</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>2042</v>
       </c>
       <c r="B26" s="10">
         <v>4310000000000</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C26" s="13">
+        <f t="shared" si="0"/>
+        <v>1.9414414414414414</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>2043</v>
       </c>
       <c r="B27" s="10">
         <v>4440000000000</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C27" s="13">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>2044</v>
       </c>
       <c r="B28" s="10">
         <v>4570000000000</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C28" s="13">
+        <f t="shared" si="0"/>
+        <v>2.0585585585585586</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>2045</v>
       </c>
       <c r="B29" s="10">
         <v>4700000000000</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C29" s="13">
+        <f t="shared" si="0"/>
+        <v>2.1171171171171173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="9">
         <v>2046</v>
       </c>
       <c r="B30" s="10">
         <v>4830000000000</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C30" s="13">
+        <f t="shared" si="0"/>
+        <v>2.1756756756756759</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="9">
         <v>2047</v>
       </c>
       <c r="B31" s="10">
         <v>4960000000000</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C31" s="13">
+        <f t="shared" si="0"/>
+        <v>2.2342342342342341</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="9">
         <v>2048</v>
       </c>
       <c r="B32" s="10">
         <v>5100000000000</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C32" s="13">
+        <f t="shared" si="0"/>
+        <v>2.2972972972972974</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>2049</v>
       </c>
       <c r="B33" s="10">
         <v>5230000000000</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C33" s="13">
+        <f t="shared" si="0"/>
+        <v>2.355855855855856</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="9">
         <v>2050</v>
       </c>
       <c r="B34" s="10">
         <v>5370000000000</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C34" s="13">
+        <f t="shared" si="0"/>
+        <v>2.4189189189189189</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="9">
         <v>2051</v>
       </c>
       <c r="B35" s="10">
         <v>5510000000000</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C35" s="13">
+        <f t="shared" si="0"/>
+        <v>2.4819819819819822</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="9">
         <v>2052</v>
       </c>
       <c r="B36" s="10">
         <v>5650000000000</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C36" s="13">
+        <f t="shared" si="0"/>
+        <v>2.545045045045045</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="9">
         <v>2053</v>
       </c>
       <c r="B37" s="10">
         <v>5790000000000</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C37" s="13">
+        <f t="shared" si="0"/>
+        <v>2.6081081081081079</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="9">
         <v>2054</v>
       </c>
       <c r="B38" s="10">
         <v>5930000000000</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C38" s="13">
+        <f t="shared" si="0"/>
+        <v>2.6711711711711712</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="9">
         <v>2055</v>
       </c>
       <c r="B39" s="10">
         <v>6060000000000</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C39" s="13">
+        <f t="shared" si="0"/>
+        <v>2.7297297297297298</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="9">
         <v>2056</v>
       </c>
       <c r="B40" s="10">
         <v>6200000000000</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C40" s="13">
+        <f t="shared" si="0"/>
+        <v>2.7927927927927927</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="9">
         <v>2057</v>
       </c>
       <c r="B41" s="10">
         <v>6340000000000</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C41" s="13">
+        <f t="shared" si="0"/>
+        <v>2.855855855855856</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="9">
         <v>2058</v>
       </c>
       <c r="B42" s="10">
         <v>6480000000000</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C42" s="13">
+        <f t="shared" si="0"/>
+        <v>2.9189189189189189</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="9">
         <v>2059</v>
       </c>
       <c r="B43" s="10">
         <v>6620000000000</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C43" s="13">
+        <f t="shared" si="0"/>
+        <v>2.9819819819819822</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="9">
         <v>2060</v>
       </c>
       <c r="B44" s="10">
         <v>6760000000000</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C44" s="13">
+        <f t="shared" si="0"/>
+        <v>3.045045045045045</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="8"/>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="8"/>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="8"/>
     </row>
   </sheetData>
@@ -922,6 +1148,116 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4F1BB5A-D768-4087-8392-4CD779301F86}">
+  <dimension ref="A3:C11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="14">
+        <v>2020</v>
+      </c>
+      <c r="B7" s="15">
+        <v>1170944075446.259</v>
+      </c>
+      <c r="C7" s="15">
+        <f>B7*About!$A$15</f>
+        <v>1134271946982.7415</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="12">
+        <v>2021</v>
+      </c>
+      <c r="B8">
+        <v>1241768434200.3643</v>
+      </c>
+      <c r="C8">
+        <f>B8*About!$A$15</f>
+        <v>1202878198111.5212</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="12">
+        <v>2022</v>
+      </c>
+      <c r="B9">
+        <v>1287835026749.8125</v>
+      </c>
+      <c r="C9">
+        <f>B9*About!$A$15</f>
+        <v>1247502057369.7097</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="12">
+        <v>2023</v>
+      </c>
+      <c r="B10">
+        <v>1331023107619.6343</v>
+      </c>
+      <c r="C10">
+        <f>B10*About!$A$15</f>
+        <v>1289337555410.8875</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="12">
+        <v>2024</v>
+      </c>
+      <c r="B11">
+        <v>1350022500028.8057</v>
+      </c>
+      <c r="C11">
+        <f>B11*About!$A$15</f>
+        <v>1307741916704.7664</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
@@ -936,10 +1272,10 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="D1" s="1"/>
     </row>
@@ -948,8 +1284,8 @@
         <v>2020</v>
       </c>
       <c r="B2" s="11">
-        <f>'OECD Data MEX'!B4*About!$A$15</f>
-        <v>2150473088428.2563</v>
+        <f>'world bank data'!C7</f>
+        <v>1134271946982.7415</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -957,8 +1293,8 @@
         <v>2021</v>
       </c>
       <c r="B3" s="11">
-        <f>'OECD Data MEX'!B5*About!$A$15</f>
-        <v>2276401692705.5864</v>
+        <f>$B$2*'OECD Data MEX'!C5</f>
+        <v>1200693277211.4607</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -966,8 +1302,8 @@
         <v>2022</v>
       </c>
       <c r="B4" s="11">
-        <f>'OECD Data MEX'!B6*About!$A$15</f>
-        <v>2373269849841.9946</v>
+        <f>$B$2*'OECD Data MEX'!C6</f>
+        <v>1251786608156.6292</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -975,8 +1311,8 @@
         <v>2023</v>
       </c>
       <c r="B5" s="11">
-        <f>'OECD Data MEX'!B7*About!$A$15</f>
-        <v>2450764375551.1211</v>
+        <f>$B$2*'OECD Data MEX'!C7</f>
+        <v>1292661272912.7639</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -984,8 +1320,8 @@
         <v>2024</v>
       </c>
       <c r="B6" s="11">
-        <f>'OECD Data MEX'!B8*About!$A$15</f>
-        <v>2508885269832.9658</v>
+        <f>$B$2*'OECD Data MEX'!C8</f>
+        <v>1323317271479.8652</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -993,8 +1329,8 @@
         <v>2025</v>
       </c>
       <c r="B7" s="11">
-        <f>'OECD Data MEX'!B9*About!$A$15</f>
-        <v>2567006164114.8105</v>
+        <f>$B$2*'OECD Data MEX'!C9</f>
+        <v>1353973270046.9661</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1002,8 +1338,8 @@
         <v>2026</v>
       </c>
       <c r="B8" s="11">
-        <f>'OECD Data MEX'!B10*About!$A$15</f>
-        <v>2625127058396.6553</v>
+        <f>$B$2*'OECD Data MEX'!C10</f>
+        <v>1384629268614.0671</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1011,8 +1347,8 @@
         <v>2027</v>
       </c>
       <c r="B9" s="11">
-        <f>'OECD Data MEX'!B11*About!$A$15</f>
-        <v>2702621584105.7817</v>
+        <f>$B$2*'OECD Data MEX'!C11</f>
+        <v>1425503933370.2021</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1020,8 +1356,8 @@
         <v>2028</v>
       </c>
       <c r="B10" s="11">
-        <f>'OECD Data MEX'!B12*About!$A$15</f>
-        <v>2770429294101.2671</v>
+        <f>$B$2*'OECD Data MEX'!C12</f>
+        <v>1461269265031.8201</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1029,8 +1365,8 @@
         <v>2029</v>
       </c>
       <c r="B11" s="11">
-        <f>'OECD Data MEX'!B13*About!$A$15</f>
-        <v>2847923819810.3936</v>
+        <f>$B$2*'OECD Data MEX'!C13</f>
+        <v>1502143929787.9548</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1038,8 +1374,8 @@
         <v>2030</v>
       </c>
       <c r="B12" s="11">
-        <f>'OECD Data MEX'!B14*About!$A$15</f>
-        <v>2935105161233.1606</v>
+        <f>$B$2*'OECD Data MEX'!C14</f>
+        <v>1548127927638.6067</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1047,8 +1383,8 @@
         <v>2031</v>
       </c>
       <c r="B13" s="11">
-        <f>'OECD Data MEX'!B15*About!$A$15</f>
-        <v>3022286502655.9277</v>
+        <f>$B$2*'OECD Data MEX'!C15</f>
+        <v>1594111925489.2583</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1056,8 +1392,8 @@
         <v>2032</v>
       </c>
       <c r="B14" s="11">
-        <f>'OECD Data MEX'!B16*About!$A$15</f>
-        <v>3109467844078.6948</v>
+        <f>$B$2*'OECD Data MEX'!C16</f>
+        <v>1640095923339.9102</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1065,8 +1401,8 @@
         <v>2033</v>
       </c>
       <c r="B15" s="11">
-        <f>'OECD Data MEX'!B17*About!$A$15</f>
-        <v>3196649185501.4619</v>
+        <f>$B$2*'OECD Data MEX'!C17</f>
+        <v>1686079921190.5615</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1074,8 +1410,8 @@
         <v>2034</v>
       </c>
       <c r="B16" s="11">
-        <f>'OECD Data MEX'!B18*About!$A$15</f>
-        <v>3293517342637.8701</v>
+        <f>$B$2*'OECD Data MEX'!C18</f>
+        <v>1737173252135.73</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -1083,8 +1419,8 @@
         <v>2035</v>
       </c>
       <c r="B17" s="11">
-        <f>'OECD Data MEX'!B19*About!$A$15</f>
-        <v>3400072315487.9185</v>
+        <f>$B$2*'OECD Data MEX'!C19</f>
+        <v>1793375916175.4155</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -1092,8 +1428,8 @@
         <v>2036</v>
       </c>
       <c r="B18" s="11">
-        <f>'OECD Data MEX'!B20*About!$A$15</f>
-        <v>3496940472624.3267</v>
+        <f>$B$2*'OECD Data MEX'!C20</f>
+        <v>1844469247120.5842</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -1101,8 +1437,8 @@
         <v>2037</v>
       </c>
       <c r="B19" s="11">
-        <f>'OECD Data MEX'!B21*About!$A$15</f>
-        <v>3603495445474.3755</v>
+        <f>$B$2*'OECD Data MEX'!C21</f>
+        <v>1900671911160.2695</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -1110,8 +1446,8 @@
         <v>2038</v>
       </c>
       <c r="B20" s="11">
-        <f>'OECD Data MEX'!B22*About!$A$15</f>
-        <v>3719737234038.0649</v>
+        <f>$B$2*'OECD Data MEX'!C22</f>
+        <v>1961983908294.4719</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -1119,8 +1455,8 @@
         <v>2039</v>
       </c>
       <c r="B21" s="11">
-        <f>'OECD Data MEX'!B23*About!$A$15</f>
-        <v>3826292206888.1138</v>
+        <f>$B$2*'OECD Data MEX'!C23</f>
+        <v>2018186572334.1572</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -1128,8 +1464,8 @@
         <v>2040</v>
       </c>
       <c r="B22" s="11">
-        <f>'OECD Data MEX'!B24*About!$A$15</f>
-        <v>3942533995451.8032</v>
+        <f>$B$2*'OECD Data MEX'!C24</f>
+        <v>2079498569468.3591</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -1137,8 +1473,8 @@
         <v>2041</v>
       </c>
       <c r="B23" s="11">
-        <f>'OECD Data MEX'!B25*About!$A$15</f>
-        <v>4058775784015.4927</v>
+        <f>$B$2*'OECD Data MEX'!C25</f>
+        <v>2140810566602.5615</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -1146,8 +1482,8 @@
         <v>2042</v>
       </c>
       <c r="B24" s="11">
-        <f>'OECD Data MEX'!B26*About!$A$15</f>
-        <v>4175017572579.1821</v>
+        <f>$B$2*'OECD Data MEX'!C26</f>
+        <v>2202122563736.7637</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -1155,8 +1491,8 @@
         <v>2043</v>
       </c>
       <c r="B25" s="11">
-        <f>'OECD Data MEX'!B27*About!$A$15</f>
-        <v>4300946176856.5127</v>
+        <f>$B$2*'OECD Data MEX'!C27</f>
+        <v>2268543893965.4829</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -1164,8 +1500,8 @@
         <v>2044</v>
       </c>
       <c r="B26" s="11">
-        <f>'OECD Data MEX'!B28*About!$A$15</f>
-        <v>4426874781133.8428</v>
+        <f>$B$2*'OECD Data MEX'!C28</f>
+        <v>2334965224194.2021</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -1173,8 +1509,8 @@
         <v>2045</v>
       </c>
       <c r="B27" s="11">
-        <f>'OECD Data MEX'!B29*About!$A$15</f>
-        <v>4552803385411.1729</v>
+        <f>$B$2*'OECD Data MEX'!C29</f>
+        <v>2401386554422.9214</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -1182,8 +1518,8 @@
         <v>2046</v>
       </c>
       <c r="B28" s="11">
-        <f>'OECD Data MEX'!B30*About!$A$15</f>
-        <v>4678731989688.5039</v>
+        <f>$B$2*'OECD Data MEX'!C30</f>
+        <v>2467807884651.6406</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -1191,8 +1527,8 @@
         <v>2047</v>
       </c>
       <c r="B29" s="11">
-        <f>'OECD Data MEX'!B31*About!$A$15</f>
-        <v>4804660593965.834</v>
+        <f>$B$2*'OECD Data MEX'!C31</f>
+        <v>2534229214880.3589</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -1200,8 +1536,8 @@
         <v>2048</v>
       </c>
       <c r="B30" s="11">
-        <f>'OECD Data MEX'!B32*About!$A$15</f>
-        <v>4940276013956.8047</v>
+        <f>$B$2*'OECD Data MEX'!C32</f>
+        <v>2605759878203.5952</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -1209,8 +1545,8 @@
         <v>2049</v>
       </c>
       <c r="B31" s="11">
-        <f>'OECD Data MEX'!B33*About!$A$15</f>
-        <v>5066204618234.1348</v>
+        <f>$B$2*'OECD Data MEX'!C33</f>
+        <v>2672181208432.3145</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -1218,8 +1554,8 @@
         <v>2050</v>
       </c>
       <c r="B32" s="11">
-        <f>'OECD Data MEX'!B34*About!$A$15</f>
-        <v>5201820038225.1064</v>
+        <f>$B$2*'OECD Data MEX'!C34</f>
+        <v>2743711871755.5503</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1227,8 +1563,8 @@
         <v>2051</v>
       </c>
       <c r="B33" s="11">
-        <f>'OECD Data MEX'!B35*About!$A$15</f>
-        <v>5337435458216.0771</v>
+        <f>$B$2*'OECD Data MEX'!C35</f>
+        <v>2815242535078.7866</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1236,8 +1572,8 @@
         <v>2052</v>
       </c>
       <c r="B34" s="11">
-        <f>'OECD Data MEX'!B36*About!$A$15</f>
-        <v>5473050878207.0488</v>
+        <f>$B$2*'OECD Data MEX'!C36</f>
+        <v>2886773198402.022</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1245,8 +1581,8 @@
         <v>2053</v>
       </c>
       <c r="B35" s="11">
-        <f>'OECD Data MEX'!B37*About!$A$15</f>
-        <v>5608666298198.0195</v>
+        <f>$B$2*'OECD Data MEX'!C37</f>
+        <v>2958303861725.2578</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1254,8 +1590,8 @@
         <v>2054</v>
       </c>
       <c r="B36" s="11">
-        <f>'OECD Data MEX'!B38*About!$A$15</f>
-        <v>5744281718188.9912</v>
+        <f>$B$2*'OECD Data MEX'!C38</f>
+        <v>3029834525048.4941</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1263,8 +1599,8 @@
         <v>2055</v>
       </c>
       <c r="B37" s="11">
-        <f>'OECD Data MEX'!B39*About!$A$15</f>
-        <v>5870210322466.3213</v>
+        <f>$B$2*'OECD Data MEX'!C39</f>
+        <v>3096255855277.2134</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1272,8 +1608,8 @@
         <v>2056</v>
       </c>
       <c r="B38" s="11">
-        <f>'OECD Data MEX'!B40*About!$A$15</f>
-        <v>6005825742457.292</v>
+        <f>$B$2*'OECD Data MEX'!C40</f>
+        <v>3167786518600.4492</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1281,8 +1617,8 @@
         <v>2057</v>
       </c>
       <c r="B39" s="11">
-        <f>'OECD Data MEX'!B41*About!$A$15</f>
-        <v>6141441162448.2637</v>
+        <f>$B$2*'OECD Data MEX'!C41</f>
+        <v>3239317181923.6851</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1290,8 +1626,8 @@
         <v>2058</v>
       </c>
       <c r="B40" s="11">
-        <f>'OECD Data MEX'!B42*About!$A$15</f>
-        <v>6277056582439.2344</v>
+        <f>$B$2*'OECD Data MEX'!C42</f>
+        <v>3310847845246.9209</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1299,8 +1635,8 @@
         <v>2059</v>
       </c>
       <c r="B41" s="11">
-        <f>'OECD Data MEX'!B43*About!$A$15</f>
-        <v>6412672002430.2061</v>
+        <f>$B$2*'OECD Data MEX'!C43</f>
+        <v>3382378508570.1572</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1308,8 +1644,8 @@
         <v>2060</v>
       </c>
       <c r="B42" s="11">
-        <f>'OECD Data MEX'!B44*About!$A$15</f>
-        <v>6548287422421.1768</v>
+        <f>$B$2*'OECD Data MEX'!C44</f>
+        <v>3453909171893.3931</v>
       </c>
       <c r="C42" s="11"/>
     </row>
@@ -1317,90 +1653,90 @@
       <c r="A43">
         <v>2061</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="16">
         <f>_xlfn.FORECAST.LINEAR(A43,$B$32:$B$42,$A$32:$A$42)</f>
-        <v>6680380363970.8125</v>
+        <v>3523581895909.5313</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2062</v>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="16">
         <f t="shared" ref="B44:B52" si="0">_xlfn.FORECAST.LINEAR(A44,$B$32:$B$42,$A$32:$A$42)</f>
-        <v>6814674854546.3125</v>
+        <v>3594415831992.5938</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2063</v>
       </c>
-      <c r="B45" s="11">
-        <f t="shared" si="0"/>
-        <v>6948969345121.7813</v>
+      <c r="B45" s="16">
+        <f t="shared" si="0"/>
+        <v>3665249768075.6875</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2064</v>
       </c>
-      <c r="B46" s="11">
-        <f t="shared" si="0"/>
-        <v>7083263835697.25</v>
+      <c r="B46" s="16">
+        <f t="shared" si="0"/>
+        <v>3736083704158.75</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2065</v>
       </c>
-      <c r="B47" s="11">
-        <f t="shared" si="0"/>
-        <v>7217558326272.7188</v>
+      <c r="B47" s="16">
+        <f t="shared" si="0"/>
+        <v>3806917640241.8438</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2066</v>
       </c>
-      <c r="B48" s="11">
-        <f t="shared" si="0"/>
-        <v>7351852816848.1875</v>
+      <c r="B48" s="16">
+        <f t="shared" si="0"/>
+        <v>3877751576324.9063</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2067</v>
       </c>
-      <c r="B49" s="11">
-        <f t="shared" si="0"/>
-        <v>7486147307423.6875</v>
+      <c r="B49" s="16">
+        <f t="shared" si="0"/>
+        <v>3948585512407.9688</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2068</v>
       </c>
-      <c r="B50" s="11">
-        <f t="shared" si="0"/>
-        <v>7620441797999.1563</v>
+      <c r="B50" s="16">
+        <f t="shared" si="0"/>
+        <v>4019419448491.0625</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2069</v>
       </c>
-      <c r="B51" s="11">
-        <f t="shared" si="0"/>
-        <v>7754736288574.625</v>
+      <c r="B51" s="16">
+        <f t="shared" si="0"/>
+        <v>4090253384574.125</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2070</v>
       </c>
-      <c r="B52" s="11">
-        <f t="shared" si="0"/>
-        <v>7889030779150.0938</v>
+      <c r="B52" s="16">
+        <f t="shared" si="0"/>
+        <v>4161087320657.1875</v>
       </c>
     </row>
   </sheetData>
@@ -1410,12 +1746,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -1559,6 +1889,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1569,15 +1905,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE6D3E8B-8F8E-4368-804E-DD1D5AFAB5A0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00BAFCA2-0CE9-422F-9C1B-DEF4BBE45CA3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1595,6 +1922,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE6D3E8B-8F8E-4368-804E-DD1D5AFAB5A0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA328D08-A500-4F74-8EC4-7A4A83520018}">
   <ds:schemaRefs>

</xml_diff>